<commit_message>
fix: distinguish source retrieval dates from unrecorded profile verification
</commit_message>
<xml_diff>
--- a/site/exports/bit-cs-image-perception.xlsx
+++ b/site/exports/bit-cs-image-perception.xlsx
@@ -452,8 +452,8 @@
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="18.2" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="37.8" customWidth="1" min="7" max="7"/>
+    <col width="26.6" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
@@ -482,7 +482,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>核对日期</t>
+          <t>已记录来源检索日期</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -549,12 +549,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>分批核实资料，不是完整名录</t>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>公开个人页（时效以核对日为准）</t>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -602,12 +602,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>分批核实资料，不是完整名录</t>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>公开个人页（时效以核对日为准）</t>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -655,12 +655,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>分批核实资料，不是完整名录</t>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>公开个人页（时效以核对日为准）</t>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>未单独记录</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>未单独记录</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">

</xml_diff>